<commit_message>
docs: sync all documentation to v5.1.4 and regenerate PDFs
</commit_message>
<xml_diff>
--- a/docs/electrical/wiring/Cable_Color_Code.xlsx
+++ b/docs/electrical/wiring/Cable_Color_Code.xlsx
@@ -32,9 +32,6 @@
     <t>TIP</t>
   </si>
   <si>
-    <t>MID</t>
-  </si>
-  <si>
     <t>REF</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>BRN (DRDY_TIP)</t>
   </si>
   <si>
-    <t>ORG/WHT (DRDY_MID)</t>
-  </si>
-  <si>
     <t>BRN/WHT (DRDY_REF)</t>
   </si>
   <si>
@@ -140,9 +134,6 @@
     <t>DRDY_REF</t>
   </si>
   <si>
-    <t>DRDY_MID</t>
-  </si>
-  <si>
     <t>Function</t>
   </si>
   <si>
@@ -159,6 +150,15 @@
   </si>
   <si>
     <t>IO01</t>
+  </si>
+  <si>
+    <t>DRDY_NEAR</t>
+  </si>
+  <si>
+    <t>NEAR</t>
+  </si>
+  <si>
+    <t>ORG/WHT (DRDY_NEAR)</t>
   </si>
 </sst>
 </file>
@@ -496,104 +496,104 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -601,33 +601,33 @@
         <v>0</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" t="s">
         <v>21</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>22</v>
-      </c>
-      <c r="E12" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -635,16 +635,16 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" t="s">
         <v>24</v>
       </c>
-      <c r="D14" t="s">
-        <v>25</v>
-      </c>
       <c r="E14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -652,16 +652,16 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -669,16 +669,16 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" t="s">
         <v>24</v>
-      </c>
-      <c r="D16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -686,16 +686,16 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -703,16 +703,16 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -720,16 +720,16 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -737,16 +737,16 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s">
         <v>26</v>
-      </c>
-      <c r="D20" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -754,16 +754,16 @@
         <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>